<commit_message>
[+] Ajout Aperçu DOB finance [~] Dernières petites modifications
</commit_message>
<xml_diff>
--- a/data/finances.xlsx
+++ b/data/finances.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="convention" sheetId="1" state="visible" r:id="rId3"/>
@@ -13,7 +13,7 @@
     <sheet name="projets" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="agents" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="budget" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="occupation" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="dob" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="67">
   <si>
     <t xml:space="preserve">cle</t>
   </si>
@@ -213,46 +213,19 @@
     <t xml:space="preserve">Formation</t>
   </si>
   <si>
-    <t xml:space="preserve">mois</t>
-  </si>
-  <si>
-    <t xml:space="preserve">taux</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fév</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Avr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Juin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jul</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aoû</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sep</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nov</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Déc</t>
+    <t xml:space="preserve">url</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://youtube.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">titre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apperçu DOB 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24 juillet 2026</t>
   </si>
 </sst>
 </file>
@@ -356,7 +329,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -382,10 +355,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -841,7 +810,7 @@
       <c r="F1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="5" t="s">
         <v>31</v>
       </c>
     </row>
@@ -904,7 +873,7 @@
       <c r="F4" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="G4" s="0" t="n">
+      <c r="G4" s="1" t="n">
         <v>56</v>
       </c>
     </row>
@@ -1107,109 +1076,76 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B2" s="1" t="s">
         <v>63</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="B2" s="1" t="n">
-        <v>60</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="B3" s="1" t="n">
+        <v>64</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="B4" s="1" t="n">
-        <v>67</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="B5" s="1" t="n">
-        <v>63</v>
-      </c>
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="B6" s="1" t="n">
-        <v>68</v>
-      </c>
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B7" s="1" t="n">
-        <v>74</v>
-      </c>
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B8" s="1" t="n">
-        <v>68</v>
-      </c>
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="B9" s="1" t="n">
-        <v>73</v>
-      </c>
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="B10" s="1" t="n">
-        <v>47</v>
-      </c>
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="B11" s="1" t="n">
-        <v>63</v>
-      </c>
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="B12" s="1" t="n">
-        <v>53</v>
-      </c>
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="B13" s="1" t="n">
-        <v>51</v>
-      </c>
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" display="https://youtube.com"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>